<commit_message>
Actualizar inventario (20 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -1,14 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB57383C-C330-4469-92F2-C8F787DD7184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Inventario" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Resumen" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Instrucciones" state="visible" r:id="rId6"/>
+    <sheet name="Inventario" sheetId="1" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" r:id="rId2"/>
+    <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -348,34 +368,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot; #,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
-      <color rgb="FF6b7472"/>
       <sz val="9"/>
+      <color rgb="FF6B7472"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -388,14 +408,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="8"/>
       <color rgb="FF9A9A9A"/>
-      <sz val="8"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -408,20 +428,20 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="9"/>
       <color rgb="FF9A9A9A"/>
-      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="15"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="15"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF2E8B80"/>
-      <sz val="11"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -472,12 +492,6 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -508,7 +522,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -524,6 +537,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -531,11 +551,21 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF6B7472"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFEDEDED"/>
         </patternFill>
       </fill>
     </dxf>
@@ -551,21 +581,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF6b7472"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFEDEDED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -903,12 +923,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H31"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -919,867 +939,948 @@
     <col min="7" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+    </row>
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+    </row>
+    <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="5">
         <v>170000</v>
       </c>
-      <c r="E5" s="8">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="10">
-        <f>IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H5" s="11" t="s">
+      <c r="E5" s="6">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="8" t="str">
+        <f t="shared" ref="G5:G31" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+    <row r="6" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="5">
         <v>130000</v>
       </c>
-      <c r="E6" s="8">
-        <v>0</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="10">
-        <f>IF(F6="NO","Oculto",IF(E6&lt;=0,"AGOTADO",IF(E6&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H6" s="11" t="s">
+      <c r="E6" s="6">
+        <v>1</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="5">
         <v>120000</v>
       </c>
-      <c r="E7" s="8">
-        <v>0</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="10">
-        <f>IF(F7="NO","Oculto",IF(E7&lt;=0,"AGOTADO",IF(E7&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H7" s="11" t="s">
+      <c r="E7" s="6">
+        <v>1</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="5">
         <v>130000</v>
       </c>
-      <c r="E8" s="8">
-        <v>0</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="10">
-        <f>IF(F8="NO","Oculto",IF(E8&lt;=0,"AGOTADO",IF(E8&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H8" s="11" t="s">
+      <c r="E8" s="6">
+        <v>1</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="5">
         <v>160000</v>
       </c>
-      <c r="E9" s="8">
-        <v>0</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="10">
-        <f>IF(F9="NO","Oculto",IF(E9&lt;=0,"AGOTADO",IF(E9&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H9" s="11" t="s">
+      <c r="E9" s="6">
+        <v>1</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+    <row r="10" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="5">
         <v>130000</v>
       </c>
-      <c r="E10" s="8">
-        <v>0</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="10">
-        <f>IF(F10="NO","Oculto",IF(E10&lt;=0,"AGOTADO",IF(E10&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H10" s="11" t="s">
+      <c r="E10" s="6">
+        <v>1</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="5">
         <v>120000</v>
       </c>
-      <c r="E11" s="8">
-        <v>0</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="10">
-        <f>IF(F11="NO","Oculto",IF(E11&lt;=0,"AGOTADO",IF(E11&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H11" s="11" t="s">
+      <c r="E11" s="6">
+        <v>1</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+    <row r="12" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="5">
         <v>160000</v>
       </c>
-      <c r="E12" s="8">
-        <v>0</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="10">
-        <f>IF(F12="NO","Oculto",IF(E12&lt;=0,"AGOTADO",IF(E12&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H12" s="11" t="s">
+      <c r="E12" s="6">
+        <v>1</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="5">
         <v>160000</v>
       </c>
-      <c r="E13" s="8">
-        <v>0</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="10">
-        <f>IF(F13="NO","Oculto",IF(E13&lt;=0,"AGOTADO",IF(E13&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H13" s="11" t="s">
+      <c r="E13" s="6">
+        <v>1</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H13" s="9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+    <row r="14" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="5">
         <v>160000</v>
       </c>
-      <c r="E14" s="8">
-        <v>0</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="10">
-        <f>IF(F14="NO","Oculto",IF(E14&lt;=0,"AGOTADO",IF(E14&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H14" s="11" t="s">
+      <c r="E14" s="6">
+        <v>1</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H14" s="9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="5">
         <v>200000</v>
       </c>
-      <c r="E15" s="8">
-        <v>0</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="10">
-        <f>IF(F15="NO","Oculto",IF(E15&lt;=0,"AGOTADO",IF(E15&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H15" s="11" t="s">
+      <c r="E15" s="6">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+    <row r="16" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="5">
         <v>130000</v>
       </c>
-      <c r="E16" s="8">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="10">
-        <f>IF(F16="NO","Oculto",IF(E16&lt;=0,"AGOTADO",IF(E16&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H16" s="11" t="s">
+      <c r="E16" s="6">
+        <v>1</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H16" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="5">
         <v>200000</v>
       </c>
-      <c r="E17" s="8">
-        <v>0</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="10">
-        <f>IF(F17="NO","Oculto",IF(E17&lt;=0,"AGOTADO",IF(E17&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H17" s="11" t="s">
+      <c r="E17" s="6">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="5">
         <v>130000</v>
       </c>
-      <c r="E18" s="8">
+      <c r="E18" s="6">
         <v>5</v>
       </c>
-      <c r="F18" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="10">
-        <f>IF(F18="NO","Oculto",IF(E18&lt;=0,"AGOTADO",IF(E18&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H18" s="11" t="s">
+      <c r="F18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H18" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="5">
         <v>120000</v>
       </c>
-      <c r="E19" s="8">
-        <v>1</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="10">
-        <f>IF(F19="NO","Oculto",IF(E19&lt;=0,"AGOTADO",IF(E19&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H19" s="11" t="s">
+      <c r="E19" s="6">
+        <v>1</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H19" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+    <row r="20" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="5">
         <v>110000</v>
       </c>
-      <c r="E20" s="8">
-        <v>0</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="10">
-        <f>IF(F20="NO","Oculto",IF(E20&lt;=0,"AGOTADO",IF(E20&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H20" s="11" t="s">
+      <c r="E20" s="6">
+        <v>1</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H20" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="5">
         <v>120000</v>
       </c>
-      <c r="E21" s="8">
-        <v>0</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="10">
-        <f>IF(F21="NO","Oculto",IF(E21&lt;=0,"AGOTADO",IF(E21&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H21" s="11" t="s">
+      <c r="E21" s="6">
+        <v>1</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H21" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+    <row r="22" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="5">
         <v>120000</v>
       </c>
-      <c r="E22" s="8">
-        <v>0</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="10">
-        <f>IF(F22="NO","Oculto",IF(E22&lt;=0,"AGOTADO",IF(E22&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H22" s="11" t="s">
+      <c r="E22" s="6">
+        <v>1</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H22" s="9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="5">
         <v>140000</v>
       </c>
-      <c r="E23" s="8">
-        <v>0</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="10">
-        <f>IF(F23="NO","Oculto",IF(E23&lt;=0,"AGOTADO",IF(E23&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H23" s="11" t="s">
+      <c r="E23" s="6">
+        <v>1</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
+    <row r="24" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="5">
         <v>130000</v>
       </c>
-      <c r="E24" s="8">
-        <v>0</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="10">
-        <f>IF(F24="NO","Oculto",IF(E24&lt;=0,"AGOTADO",IF(E24&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H24" s="11" t="s">
+      <c r="E24" s="6">
+        <v>1</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H24" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="5">
         <v>130000</v>
       </c>
-      <c r="E25" s="8">
-        <v>0</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="10">
-        <f>IF(F25="NO","Oculto",IF(E25&lt;=0,"AGOTADO",IF(E25&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H25" s="11" t="s">
+      <c r="E25" s="6">
+        <v>1</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
+    <row r="26" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="5">
         <v>140000</v>
       </c>
-      <c r="E26" s="8">
-        <v>5</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="10">
-        <f>IF(F26="NO","Oculto",IF(E26&lt;=0,"AGOTADO",IF(E26&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H26" s="11" t="s">
+      <c r="E26" s="6">
+        <v>1</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H26" s="9" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="5">
         <v>130000</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="6">
         <v>2</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="10">
-        <f>IF(F27="NO","Oculto",IF(E27&lt;=0,"AGOTADO",IF(E27&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H27" s="11" t="s">
+      <c r="F27" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H27" s="9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
+    <row r="28" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="5">
         <v>120000</v>
       </c>
-      <c r="E28" s="8">
-        <v>1</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="10">
-        <f>IF(F28="NO","Oculto",IF(E28&lt;=0,"AGOTADO",IF(E28&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H28" s="11" t="s">
+      <c r="E28" s="6">
+        <v>1</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H28" s="9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="5">
         <v>140000</v>
       </c>
-      <c r="E29" s="8">
-        <v>1</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="10">
-        <f>IF(F29="NO","Oculto",IF(E29&lt;=0,"AGOTADO",IF(E29&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H29" s="11" t="s">
+      <c r="E29" s="6">
+        <v>1</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
+    <row r="30" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="5">
         <v>160000</v>
       </c>
-      <c r="E30" s="8">
-        <v>1</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="10">
-        <f>IF(F30="NO","Oculto",IF(E30&lt;=0,"AGOTADO",IF(E30&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H30" s="11" t="s">
+      <c r="E30" s="6">
+        <v>1</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H30" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
+    <row r="31" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="5">
         <v>60000</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31" s="6">
         <v>10</v>
       </c>
-      <c r="F31" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="10">
-        <f>IF(F31="NO","Oculto",IF(E31&lt;=0,"AGOTADO",IF(E31&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H31" s="11" t="s">
+      <c r="F31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Disponible</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>77</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G31"/>
+  <autoFilter ref="A4:G31" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G31">
-    <cfRule type="containsText" dxfId="0" priority="1">
-      <formula>NOT(ISERROR(SEARCH("AGOTADO",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2">
-      <formula>NOT(ISERROR(SEARCH("Últimas",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3">
-      <formula>NOT(ISERROR(SEARCH("Oculto",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4">
-      <formula>NOT(ISERROR(SEARCH("Disponible",G5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E31">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E31" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F31">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F31" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{00000000-000E-0000-0000-000001000000}">
+            <xm:f>NOT(ISERROR(SEARCH("AGOTADO",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{00000000-000E-0000-0000-000002000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Últimas",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C6500"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{00000000-000E-0000-0000-000003000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Oculto",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF6B7472"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFEDEDED"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{00000000-000E-0000-0000-000004000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Disponible",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>G5:G31</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="13"/>
+      <c r="B1" s="20"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="12">
         <f>COUNTA(Inventario!$A$5:$A$31)</f>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$31,"Disponible")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$31,"Últimas unidades")</f>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$31,"AGOTADO")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$31,"Oculto")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="12">
         <f>SUM(Inventario!$E$5:$E$31)</f>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="13">
         <f>SUMPRODUCT(Inventario!$D$5:$D$31,Inventario!$E$5:$E$31)</f>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+        <v>4910000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="14" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1788,145 +1889,145 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="10" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="10" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="17" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="10" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="10" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="10" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="10" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="17" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="10" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="10" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="10" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="10" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="10" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="17" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="10" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="10" t="s">
         <v>109</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar inventario (24 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB57383C-C330-4469-92F2-C8F787DD7184}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D03597-617F-43DF-9F22-BB593D4A7A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1001,14 +1001,14 @@
         <v>170000</v>
       </c>
       <c r="E5" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="8" t="str">
         <f t="shared" ref="G5:G31" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>14</v>
@@ -1028,14 +1028,14 @@
         <v>130000</v>
       </c>
       <c r="E6" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H6" s="9" t="s">
         <v>17</v>
@@ -1055,14 +1055,14 @@
         <v>120000</v>
       </c>
       <c r="E7" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>20</v>
@@ -1082,14 +1082,14 @@
         <v>130000</v>
       </c>
       <c r="E8" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>23</v>
@@ -1109,14 +1109,14 @@
         <v>160000</v>
       </c>
       <c r="E9" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H9" s="9" t="s">
         <v>25</v>
@@ -1136,14 +1136,14 @@
         <v>130000</v>
       </c>
       <c r="E10" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>27</v>
@@ -1163,14 +1163,14 @@
         <v>120000</v>
       </c>
       <c r="E11" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>29</v>
@@ -1190,14 +1190,14 @@
         <v>160000</v>
       </c>
       <c r="E12" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F12" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H12" s="9" t="s">
         <v>33</v>
@@ -1217,14 +1217,14 @@
         <v>160000</v>
       </c>
       <c r="E13" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>35</v>
@@ -1244,14 +1244,14 @@
         <v>160000</v>
       </c>
       <c r="E14" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G14" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H14" s="9" t="s">
         <v>37</v>
@@ -1271,14 +1271,14 @@
         <v>200000</v>
       </c>
       <c r="E15" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F15" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G15" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>39</v>
@@ -1298,14 +1298,14 @@
         <v>130000</v>
       </c>
       <c r="E16" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>41</v>
@@ -1325,14 +1325,14 @@
         <v>200000</v>
       </c>
       <c r="E17" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G17" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>43</v>
@@ -1352,14 +1352,14 @@
         <v>130000</v>
       </c>
       <c r="E18" s="6">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>45</v>
@@ -1379,14 +1379,14 @@
         <v>120000</v>
       </c>
       <c r="E19" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H19" s="9" t="s">
         <v>47</v>
@@ -1406,14 +1406,14 @@
         <v>110000</v>
       </c>
       <c r="E20" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G20" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>49</v>
@@ -1433,14 +1433,14 @@
         <v>120000</v>
       </c>
       <c r="E21" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F21" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G21" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H21" s="9" t="s">
         <v>52</v>
@@ -1460,14 +1460,14 @@
         <v>120000</v>
       </c>
       <c r="E22" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G22" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H22" s="9" t="s">
         <v>54</v>
@@ -1487,14 +1487,14 @@
         <v>140000</v>
       </c>
       <c r="E23" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G23" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H23" s="9" t="s">
         <v>57</v>
@@ -1514,14 +1514,14 @@
         <v>130000</v>
       </c>
       <c r="E24" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G24" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>60</v>
@@ -1541,14 +1541,14 @@
         <v>130000</v>
       </c>
       <c r="E25" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>62</v>
@@ -1568,7 +1568,7 @@
         <v>140000</v>
       </c>
       <c r="E26" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>13</v>
@@ -1595,7 +1595,7 @@
         <v>130000</v>
       </c>
       <c r="E27" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" s="7" t="s">
         <v>13</v>
@@ -1676,14 +1676,14 @@
         <v>160000</v>
       </c>
       <c r="E30" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G30" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
+        <v>AGOTADO</v>
       </c>
       <c r="H30" s="9" t="s">
         <v>75</v>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="B5" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$31,"Últimas unidades")</f>
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B6" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$31,"AGOTADO")</f>
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1862,7 +1862,7 @@
       </c>
       <c r="B8" s="12">
         <f>SUM(Inventario!$E$5:$E$31)</f>
-        <v>41</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1871,7 +1871,7 @@
       </c>
       <c r="B9" s="13">
         <f>SUMPRODUCT(Inventario!$D$5:$D$31,Inventario!$E$5:$E$31)</f>
-        <v>4910000</v>
+        <v>1410000</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizar inventario (0 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -1,39 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
-  <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D03597-617F-43DF-9F22-BB593D4A7A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet name="Inventario" sheetId="1" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" r:id="rId2"/>
-    <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
+    <sheet sheetId="1" name="Inventario" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="Resumen" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Instrucciones" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="112">
   <si>
     <t>INVENTARIO — El Garaje de Rochi</t>
   </si>
@@ -269,6 +249,12 @@
     <t>CP-MINOXIDIL</t>
   </si>
   <si>
+    <t>Kirkland Glucosamina y Condroitina (280 tabletas)</t>
+  </si>
+  <si>
+    <t>SUP-GLUCO-280</t>
+  </si>
+  <si>
     <t>RESUMEN DEL INVENTARIO</t>
   </si>
   <si>
@@ -296,7 +282,7 @@
     <t>Se recalcula solo cuando cambias las cantidades en la hoja Inventario.</t>
   </si>
   <si>
-    <t>Generado: 4/8/2026, 3:25:48 p. m.</t>
+    <t>Generado: 11/8/2026, 1:14:25 p. m.</t>
   </si>
   <si>
     <t>CÓMO USAR ESTE EXCEL</t>
@@ -368,34 +354,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot; #,##0"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="16"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
+      <color rgb="FF6b7472"/>
       <sz val="9"/>
-      <color rgb="FF6B7472"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -408,14 +394,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF9A9A9A"/>
       <sz val="8"/>
-      <color rgb="FF9A9A9A"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="14"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -428,20 +414,20 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF9A9A9A"/>
       <sz val="9"/>
-      <color rgb="FF9A9A9A"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="15"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <color rgb="FF2E8B80"/>
       <sz val="11"/>
-      <color rgb="FF2E8B80"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -492,6 +478,12 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -522,6 +514,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -537,13 +530,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -551,21 +537,11 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF006100"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF6B7472"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFEDEDED"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -581,11 +557,21 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF6b7472"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFEDEDED"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -923,12 +909,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -939,949 +925,894 @@
     <col min="7" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-    </row>
-    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-    </row>
-    <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H4" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="7">
         <v>170000</v>
       </c>
-      <c r="E5" s="6">
-        <v>0</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="8" t="str">
-        <f t="shared" ref="G5:G31" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H5" s="9" t="s">
+      <c r="E5" s="8">
+        <v>0</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="10">
+        <f>IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H5" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="7">
         <v>130000</v>
       </c>
-      <c r="E6" s="6">
-        <v>0</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H6" s="9" t="s">
+      <c r="E6" s="8">
+        <v>0</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="10">
+        <f>IF(F6="NO","Oculto",IF(E6&lt;=0,"AGOTADO",IF(E6&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H6" s="11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="7">
         <v>120000</v>
       </c>
-      <c r="E7" s="6">
-        <v>0</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H7" s="9" t="s">
+      <c r="E7" s="8">
+        <v>0</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="10">
+        <f>IF(F7="NO","Oculto",IF(E7&lt;=0,"AGOTADO",IF(E7&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H7" s="11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
+    <row r="8" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="7">
         <v>130000</v>
       </c>
-      <c r="E8" s="6">
-        <v>0</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H8" s="9" t="s">
+      <c r="E8" s="8">
+        <v>0</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="10">
+        <f>IF(F8="NO","Oculto",IF(E8&lt;=0,"AGOTADO",IF(E8&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H8" s="11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="7">
         <v>160000</v>
       </c>
-      <c r="E9" s="6">
-        <v>0</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H9" s="9" t="s">
+      <c r="E9" s="8">
+        <v>0</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="10">
+        <f>IF(F9="NO","Oculto",IF(E9&lt;=0,"AGOTADO",IF(E9&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H9" s="11" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="7">
         <v>130000</v>
       </c>
-      <c r="E10" s="6">
-        <v>0</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H10" s="9" t="s">
+      <c r="E10" s="8">
+        <v>0</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="10">
+        <f>IF(F10="NO","Oculto",IF(E10&lt;=0,"AGOTADO",IF(E10&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H10" s="11" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
+    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="7">
         <v>120000</v>
       </c>
-      <c r="E11" s="6">
-        <v>0</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H11" s="9" t="s">
+      <c r="E11" s="8">
+        <v>0</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="10">
+        <f>IF(F11="NO","Oculto",IF(E11&lt;=0,"AGOTADO",IF(E11&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H11" s="11" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
+    <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="7">
         <v>160000</v>
       </c>
-      <c r="E12" s="6">
-        <v>0</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H12" s="9" t="s">
+      <c r="E12" s="8">
+        <v>0</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="10">
+        <f>IF(F12="NO","Oculto",IF(E12&lt;=0,"AGOTADO",IF(E12&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H12" s="11" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="7">
         <v>160000</v>
       </c>
-      <c r="E13" s="6">
-        <v>0</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H13" s="9" t="s">
+      <c r="E13" s="8">
+        <v>0</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="10">
+        <f>IF(F13="NO","Oculto",IF(E13&lt;=0,"AGOTADO",IF(E13&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H13" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+    <row r="14" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="7">
         <v>160000</v>
       </c>
-      <c r="E14" s="6">
-        <v>0</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H14" s="9" t="s">
+      <c r="E14" s="8">
+        <v>0</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="10">
+        <f>IF(F14="NO","Oculto",IF(E14&lt;=0,"AGOTADO",IF(E14&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H14" s="11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="7">
         <v>200000</v>
       </c>
-      <c r="E15" s="6">
-        <v>0</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H15" s="9" t="s">
+      <c r="E15" s="8">
+        <v>0</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="10">
+        <f>IF(F15="NO","Oculto",IF(E15&lt;=0,"AGOTADO",IF(E15&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H15" s="11" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="10" t="s">
+    <row r="16" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="7">
         <v>130000</v>
       </c>
-      <c r="E16" s="6">
-        <v>0</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H16" s="9" t="s">
+      <c r="E16" s="8">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="10">
+        <f>IF(F16="NO","Oculto",IF(E16&lt;=0,"AGOTADO",IF(E16&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H16" s="11" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="B17" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="7">
         <v>200000</v>
       </c>
-      <c r="E17" s="6">
-        <v>0</v>
-      </c>
-      <c r="F17" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H17" s="9" t="s">
+      <c r="E17" s="8">
+        <v>0</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="10">
+        <f>IF(F17="NO","Oculto",IF(E17&lt;=0,"AGOTADO",IF(E17&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H17" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
+    <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="7">
         <v>130000</v>
       </c>
-      <c r="E18" s="6">
-        <v>0</v>
-      </c>
-      <c r="F18" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H18" s="9" t="s">
+      <c r="E18" s="8">
+        <v>0</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="10">
+        <f>IF(F18="NO","Oculto",IF(E18&lt;=0,"AGOTADO",IF(E18&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H18" s="11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="5">
+      <c r="D19" s="7">
         <v>120000</v>
       </c>
-      <c r="E19" s="6">
-        <v>0</v>
-      </c>
-      <c r="F19" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H19" s="9" t="s">
+      <c r="E19" s="8">
+        <v>0</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="10">
+        <f>IF(F19="NO","Oculto",IF(E19&lt;=0,"AGOTADO",IF(E19&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H19" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
+    <row r="20" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="5">
+      <c r="D20" s="7">
         <v>110000</v>
       </c>
-      <c r="E20" s="6">
-        <v>0</v>
-      </c>
-      <c r="F20" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H20" s="9" t="s">
+      <c r="E20" s="8">
+        <v>0</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="10">
+        <f>IF(F20="NO","Oculto",IF(E20&lt;=0,"AGOTADO",IF(E20&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H20" s="11" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="5">
+      <c r="D21" s="7">
         <v>120000</v>
       </c>
-      <c r="E21" s="6">
-        <v>0</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H21" s="9" t="s">
+      <c r="E21" s="8">
+        <v>0</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="10">
+        <f>IF(F21="NO","Oculto",IF(E21&lt;=0,"AGOTADO",IF(E21&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H21" s="11" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
+    <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="5">
+      <c r="D22" s="7">
         <v>120000</v>
       </c>
-      <c r="E22" s="6">
-        <v>0</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H22" s="9" t="s">
+      <c r="E22" s="8">
+        <v>0</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="10">
+        <f>IF(F22="NO","Oculto",IF(E22&lt;=0,"AGOTADO",IF(E22&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H22" s="11" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    <row r="23" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="4" t="s">
+      <c r="B23" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="5">
+      <c r="D23" s="7">
         <v>140000</v>
       </c>
-      <c r="E23" s="6">
-        <v>0</v>
-      </c>
-      <c r="F23" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H23" s="9" t="s">
+      <c r="E23" s="8">
+        <v>0</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="10">
+        <f>IF(F23="NO","Oculto",IF(E23&lt;=0,"AGOTADO",IF(E23&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H23" s="11" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+    <row r="24" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="5">
+      <c r="D24" s="7">
         <v>130000</v>
       </c>
-      <c r="E24" s="6">
-        <v>0</v>
-      </c>
-      <c r="F24" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H24" s="9" t="s">
+      <c r="E24" s="8">
+        <v>0</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="10">
+        <f>IF(F24="NO","Oculto",IF(E24&lt;=0,"AGOTADO",IF(E24&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H24" s="11" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="4" t="s">
+      <c r="B25" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="5">
+      <c r="D25" s="7">
         <v>130000</v>
       </c>
-      <c r="E25" s="6">
-        <v>0</v>
-      </c>
-      <c r="F25" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H25" s="9" t="s">
+      <c r="E25" s="8">
+        <v>0</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="10">
+        <f>IF(F25="NO","Oculto",IF(E25&lt;=0,"AGOTADO",IF(E25&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H25" s="11" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+    <row r="26" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="5">
+      <c r="D26" s="7">
         <v>140000</v>
       </c>
-      <c r="E26" s="6">
+      <c r="E26" s="8">
         <v>3</v>
       </c>
-      <c r="F26" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H26" s="9" t="s">
+      <c r="F26" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="10">
+        <f>IF(F26="NO","Oculto",IF(E26&lt;=0,"AGOTADO",IF(E26&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H26" s="11" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="4" t="s">
+      <c r="C27" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D27" s="5">
+      <c r="D27" s="7">
         <v>130000</v>
       </c>
-      <c r="E27" s="6">
+      <c r="E27" s="8">
         <v>1</v>
       </c>
-      <c r="F27" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H27" s="9" t="s">
+      <c r="F27" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="10">
+        <f>IF(F27="NO","Oculto",IF(E27&lt;=0,"AGOTADO",IF(E27&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H27" s="11" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+    <row r="28" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="5">
+      <c r="D28" s="7">
         <v>120000</v>
       </c>
-      <c r="E28" s="6">
+      <c r="E28" s="8">
         <v>1</v>
       </c>
-      <c r="F28" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H28" s="9" t="s">
+      <c r="F28" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="10">
+        <f>IF(F28="NO","Oculto",IF(E28&lt;=0,"AGOTADO",IF(E28&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H28" s="11" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
+    <row r="29" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="B29" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C29" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="5">
+      <c r="D29" s="7">
         <v>140000</v>
       </c>
-      <c r="E29" s="6">
+      <c r="E29" s="8">
         <v>1</v>
       </c>
-      <c r="F29" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Últimas unidades</v>
-      </c>
-      <c r="H29" s="9" t="s">
+      <c r="F29" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="10">
+        <f>IF(F29="NO","Oculto",IF(E29&lt;=0,"AGOTADO",IF(E29&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H29" s="11" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
+    <row r="30" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="5">
+      <c r="D30" s="7">
         <v>160000</v>
       </c>
-      <c r="E30" s="6">
-        <v>0</v>
-      </c>
-      <c r="F30" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>AGOTADO</v>
-      </c>
-      <c r="H30" s="9" t="s">
+      <c r="E30" s="8">
+        <v>0</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="10">
+        <f>IF(F30="NO","Oculto",IF(E30&lt;=0,"AGOTADO",IF(E30&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H30" s="11" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C31" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="5">
+      <c r="D31" s="7">
         <v>60000</v>
       </c>
-      <c r="E31" s="6">
+      <c r="E31" s="8">
         <v>10</v>
       </c>
-      <c r="F31" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="8" t="str">
-        <f t="shared" si="0"/>
-        <v>Disponible</v>
-      </c>
-      <c r="H31" s="9" t="s">
+      <c r="F31" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="10">
+        <f>IF(F31="NO","Oculto",IF(E31&lt;=0,"AGOTADO",IF(E31&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H31" s="11" t="s">
         <v>77</v>
       </c>
     </row>
+    <row r="32" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D32" s="7">
+        <v>160000</v>
+      </c>
+      <c r="E32" s="8">
+        <v>2</v>
+      </c>
+      <c r="F32" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="10">
+        <f>IF(F32="NO","Oculto",IF(E32&lt;=0,"AGOTADO",IF(E32&lt;=5,"Últimas unidades","Disponible")))</f>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G31" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A4:G32"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
+  <conditionalFormatting sqref="G5:G32">
+    <cfRule type="containsText" dxfId="0" priority="1">
+      <formula>NOT(ISERROR(SEARCH("AGOTADO",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2">
+      <formula>NOT(ISERROR(SEARCH("Últimas",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="3">
+      <formula>NOT(ISERROR(SEARCH("Oculto",G5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="3" priority="4">
+      <formula>NOT(ISERROR(SEARCH("Disponible",G5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E31" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E32">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F31" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F32">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
-      <x14:conditionalFormattings>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{00000000-000E-0000-0000-000001000000}">
-            <xm:f>NOT(ISERROR(SEARCH("AGOTADO",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C0006"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFFFC7CE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{00000000-000E-0000-0000-000002000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Últimas",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF9C6500"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFFFEB9C"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{00000000-000E-0000-0000-000003000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Oculto",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF6B7472"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFEDEDED"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{00000000-000E-0000-0000-000004000000}">
-            <xm:f>NOT(ISERROR(SEARCH("Disponible",G5)))</xm:f>
-            <x14:dxf>
-              <font>
-                <color rgb="FF006100"/>
-              </font>
-              <fill>
-                <patternFill patternType="solid">
-                  <bgColor rgb="FFC6EFCE"/>
-                </patternFill>
-              </fill>
-            </x14:dxf>
-          </x14:cfRule>
-          <xm:sqref>G5:G31</xm:sqref>
-        </x14:conditionalFormatting>
-      </x14:conditionalFormattings>
-    </ext>
-  </extLst>
+  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="B1" s="20"/>
+    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B1" s="13"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="B3" s="12">
-        <f>COUNTA(Inventario!$A$5:$A$31)</f>
-        <v>27</v>
+      <c r="A3" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="15">
+        <f>COUNTA(Inventario!$A$5:$A$32)</f>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="B4" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$31,"Disponible")</f>
-        <v>1</v>
+      <c r="A4" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$32,"Disponible")</f>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$31,"Últimas unidades")</f>
-        <v>4</v>
+      <c r="A5" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$32,"Últimas unidades")</f>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="B6" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$31,"AGOTADO")</f>
-        <v>22</v>
+      <c r="A6" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$32,"AGOTADO")</f>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="B7" s="12">
-        <f>COUNTIF(Inventario!$G$5:$G$31,"Oculto")</f>
-        <v>0</v>
+      <c r="A7" s="14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="15">
+        <f>COUNTIF(Inventario!$G$5:$G$32,"Oculto")</f>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="12">
-        <f>SUM(Inventario!$E$5:$E$31)</f>
-        <v>16</v>
+      <c r="A8" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="B8" s="15">
+        <f>SUM(Inventario!$E$5:$E$32)</f>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="13">
-        <f>SUMPRODUCT(Inventario!$D$5:$D$31,Inventario!$E$5:$E$31)</f>
-        <v>1410000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>87</v>
+      </c>
+      <c r="B9" s="16">
+        <f>SUMPRODUCT(Inventario!$D$5:$D$32,Inventario!$E$5:$E$32)</f>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" s="18" t="s">
+        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1889,145 +1820,145 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
-        <v>88</v>
+    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="19" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>89</v>
+      <c r="A2" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
-        <v>90</v>
+      <c r="A3" s="12" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="10" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="10" t="s">
-        <v>89</v>
-      </c>
-    </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>95</v>
+      <c r="A9" s="20" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>96</v>
+      <c r="A10" s="12" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>97</v>
+      <c r="A11" s="12" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>98</v>
+      <c r="A12" s="12" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>99</v>
+      <c r="A13" s="12" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>100</v>
+      <c r="A14" s="12" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>89</v>
+      <c r="A15" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="17" t="s">
-        <v>101</v>
+      <c r="A16" s="20" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>102</v>
+      <c r="A17" s="12" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10" t="s">
-        <v>103</v>
+      <c r="A18" s="12" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>104</v>
+      <c r="A19" s="12" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="10" t="s">
-        <v>105</v>
+      <c r="A20" s="12" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>89</v>
+      <c r="A21" s="12" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="17" t="s">
-        <v>106</v>
+      <c r="A22" s="20" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>107</v>
+      <c r="A23" s="12" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>108</v>
+      <c r="A24" s="12" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>109</v>
+      <c r="A25" s="12" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar inventario (1 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -1,14 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF9245BF-17A0-4AA1-99E1-C95E3EDF9679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Inventario" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Resumen" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Instrucciones" state="visible" r:id="rId6"/>
+    <sheet name="Inventario" sheetId="1" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" r:id="rId2"/>
+    <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -354,34 +374,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot; #,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
-      <color rgb="FF6b7472"/>
       <sz val="9"/>
+      <color rgb="FF6B7472"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -394,14 +414,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="8"/>
       <color rgb="FF9A9A9A"/>
-      <sz val="8"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -414,20 +434,20 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="9"/>
       <color rgb="FF9A9A9A"/>
-      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="15"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="15"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF2E8B80"/>
-      <sz val="11"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -478,12 +498,6 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -514,7 +528,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -530,6 +543,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,11 +557,21 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF6B7472"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFEDEDED"/>
         </patternFill>
       </fill>
     </dxf>
@@ -557,21 +587,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF6b7472"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFEDEDED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -909,12 +929,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -925,893 +945,975 @@
     <col min="7" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+    </row>
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+    </row>
+    <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="5">
         <v>170000</v>
       </c>
-      <c r="E5" s="8">
-        <v>0</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="10">
-        <f>IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H5" s="11" t="s">
+      <c r="E5" s="6">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="8" t="str">
+        <f t="shared" ref="G5:G32" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+    <row r="6" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="5">
         <v>130000</v>
       </c>
-      <c r="E6" s="8">
-        <v>0</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="10">
-        <f>IF(F6="NO","Oculto",IF(E6&lt;=0,"AGOTADO",IF(E6&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H6" s="11" t="s">
+      <c r="E6" s="6">
+        <v>2</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="5">
         <v>120000</v>
       </c>
-      <c r="E7" s="8">
-        <v>0</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="10">
-        <f>IF(F7="NO","Oculto",IF(E7&lt;=0,"AGOTADO",IF(E7&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H7" s="11" t="s">
+      <c r="E7" s="6">
+        <v>0</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="5">
         <v>130000</v>
       </c>
-      <c r="E8" s="8">
-        <v>0</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="10">
-        <f>IF(F8="NO","Oculto",IF(E8&lt;=0,"AGOTADO",IF(E8&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H8" s="11" t="s">
+      <c r="E8" s="6">
+        <v>0</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="5">
         <v>160000</v>
       </c>
-      <c r="E9" s="8">
-        <v>0</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="10">
-        <f>IF(F9="NO","Oculto",IF(E9&lt;=0,"AGOTADO",IF(E9&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H9" s="11" t="s">
+      <c r="E9" s="6">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+    <row r="10" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="5">
         <v>130000</v>
       </c>
-      <c r="E10" s="8">
-        <v>0</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="10">
-        <f>IF(F10="NO","Oculto",IF(E10&lt;=0,"AGOTADO",IF(E10&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H10" s="11" t="s">
+      <c r="E10" s="6">
+        <v>0</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="5">
         <v>120000</v>
       </c>
-      <c r="E11" s="8">
-        <v>0</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="10">
-        <f>IF(F11="NO","Oculto",IF(E11&lt;=0,"AGOTADO",IF(E11&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H11" s="11" t="s">
+      <c r="E11" s="6">
+        <v>0</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H11" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+    <row r="12" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D12" s="5">
         <v>160000</v>
       </c>
-      <c r="E12" s="8">
-        <v>0</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="10">
-        <f>IF(F12="NO","Oculto",IF(E12&lt;=0,"AGOTADO",IF(E12&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H12" s="11" t="s">
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H12" s="9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D13" s="5">
         <v>160000</v>
       </c>
-      <c r="E13" s="8">
-        <v>0</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="10">
-        <f>IF(F13="NO","Oculto",IF(E13&lt;=0,"AGOTADO",IF(E13&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H13" s="11" t="s">
+      <c r="E13" s="6">
+        <v>0</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H13" s="9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+    <row r="14" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D14" s="7">
+      <c r="D14" s="5">
         <v>160000</v>
       </c>
-      <c r="E14" s="8">
-        <v>0</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="10">
-        <f>IF(F14="NO","Oculto",IF(E14&lt;=0,"AGOTADO",IF(E14&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H14" s="11" t="s">
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H14" s="9" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="7">
+      <c r="D15" s="5">
         <v>200000</v>
       </c>
-      <c r="E15" s="8">
-        <v>0</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="10">
-        <f>IF(F15="NO","Oculto",IF(E15&lt;=0,"AGOTADO",IF(E15&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H15" s="11" t="s">
+      <c r="E15" s="6">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H15" s="9" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+    <row r="16" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D16" s="7">
+      <c r="D16" s="5">
         <v>130000</v>
       </c>
-      <c r="E16" s="8">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="10">
-        <f>IF(F16="NO","Oculto",IF(E16&lt;=0,"AGOTADO",IF(E16&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H16" s="11" t="s">
+      <c r="E16" s="6">
+        <v>0</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H16" s="9" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="5">
         <v>200000</v>
       </c>
-      <c r="E17" s="8">
-        <v>0</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="10">
-        <f>IF(F17="NO","Oculto",IF(E17&lt;=0,"AGOTADO",IF(E17&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H17" s="11" t="s">
+      <c r="E17" s="6">
+        <v>0</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H17" s="9" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+    <row r="18" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="7">
+      <c r="D18" s="5">
         <v>130000</v>
       </c>
-      <c r="E18" s="8">
-        <v>0</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="10">
-        <f>IF(F18="NO","Oculto",IF(E18&lt;=0,"AGOTADO",IF(E18&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H18" s="11" t="s">
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H18" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="19" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D19" s="7">
+      <c r="D19" s="5">
         <v>120000</v>
       </c>
-      <c r="E19" s="8">
-        <v>0</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="10">
-        <f>IF(F19="NO","Oculto",IF(E19&lt;=0,"AGOTADO",IF(E19&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H19" s="11" t="s">
+      <c r="E19" s="6">
+        <v>0</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H19" s="9" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+    <row r="20" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D20" s="7">
+      <c r="D20" s="5">
         <v>110000</v>
       </c>
-      <c r="E20" s="8">
-        <v>0</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="10">
-        <f>IF(F20="NO","Oculto",IF(E20&lt;=0,"AGOTADO",IF(E20&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H20" s="11" t="s">
+      <c r="E20" s="6">
+        <v>0</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H20" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
+    <row r="21" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D21" s="7">
+      <c r="D21" s="5">
         <v>120000</v>
       </c>
-      <c r="E21" s="8">
-        <v>0</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="10">
-        <f>IF(F21="NO","Oculto",IF(E21&lt;=0,"AGOTADO",IF(E21&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H21" s="11" t="s">
+      <c r="E21" s="6">
+        <v>0</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H21" s="9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+    <row r="22" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D22" s="7">
+      <c r="D22" s="5">
         <v>120000</v>
       </c>
-      <c r="E22" s="8">
-        <v>0</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="10">
-        <f>IF(F22="NO","Oculto",IF(E22&lt;=0,"AGOTADO",IF(E22&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H22" s="11" t="s">
+      <c r="E22" s="6">
+        <v>0</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H22" s="9" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="23" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D23" s="7">
+      <c r="D23" s="5">
         <v>140000</v>
       </c>
-      <c r="E23" s="8">
-        <v>0</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="10">
-        <f>IF(F23="NO","Oculto",IF(E23&lt;=0,"AGOTADO",IF(E23&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H23" s="11" t="s">
+      <c r="E23" s="6">
+        <v>0</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H23" s="9" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
+    <row r="24" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="B24" s="4" t="s">
+      <c r="B24" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="4" t="s">
+      <c r="C24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D24" s="7">
+      <c r="D24" s="5">
         <v>130000</v>
       </c>
-      <c r="E24" s="8">
-        <v>0</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="10">
-        <f>IF(F24="NO","Oculto",IF(E24&lt;=0,"AGOTADO",IF(E24&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H24" s="11" t="s">
+      <c r="E24" s="6">
+        <v>0</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H24" s="9" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
+    <row r="25" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D25" s="7">
+      <c r="D25" s="5">
         <v>130000</v>
       </c>
-      <c r="E25" s="8">
-        <v>0</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="10">
-        <f>IF(F25="NO","Oculto",IF(E25&lt;=0,"AGOTADO",IF(E25&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H25" s="11" t="s">
+      <c r="E25" s="6">
+        <v>0</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H25" s="9" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="26" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
+    <row r="26" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="4" t="s">
+      <c r="B26" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="C26" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D26" s="7">
+      <c r="D26" s="5">
         <v>140000</v>
       </c>
-      <c r="E26" s="8">
+      <c r="E26" s="6">
         <v>3</v>
       </c>
-      <c r="F26" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="10">
-        <f>IF(F26="NO","Oculto",IF(E26&lt;=0,"AGOTADO",IF(E26&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H26" s="11" t="s">
+      <c r="F26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H26" s="9" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+    <row r="27" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D27" s="7">
+      <c r="D27" s="5">
         <v>130000</v>
       </c>
-      <c r="E27" s="8">
+      <c r="E27" s="6">
         <v>1</v>
       </c>
-      <c r="F27" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="10">
-        <f>IF(F27="NO","Oculto",IF(E27&lt;=0,"AGOTADO",IF(E27&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H27" s="11" t="s">
+      <c r="F27" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H27" s="9" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
+    <row r="28" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C28" s="4" t="s">
+      <c r="C28" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D28" s="7">
+      <c r="D28" s="5">
         <v>120000</v>
       </c>
-      <c r="E28" s="8">
+      <c r="E28" s="6">
         <v>1</v>
       </c>
-      <c r="F28" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="10">
-        <f>IF(F28="NO","Oculto",IF(E28&lt;=0,"AGOTADO",IF(E28&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H28" s="11" t="s">
+      <c r="F28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H28" s="9" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="29" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+    <row r="29" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D29" s="7">
+      <c r="D29" s="5">
         <v>140000</v>
       </c>
-      <c r="E29" s="8">
+      <c r="E29" s="6">
         <v>1</v>
       </c>
-      <c r="F29" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="10">
-        <f>IF(F29="NO","Oculto",IF(E29&lt;=0,"AGOTADO",IF(E29&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H29" s="11" t="s">
+      <c r="F29" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H29" s="9" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
+    <row r="30" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="B30" s="4" t="s">
+      <c r="B30" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="C30" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D30" s="7">
+      <c r="D30" s="5">
         <v>160000</v>
       </c>
-      <c r="E30" s="8">
-        <v>0</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="10">
-        <f>IF(F30="NO","Oculto",IF(E30&lt;=0,"AGOTADO",IF(E30&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H30" s="11" t="s">
+      <c r="E30" s="6">
+        <v>0</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H30" s="9" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
+    <row r="31" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="5">
         <v>60000</v>
       </c>
-      <c r="E31" s="8">
+      <c r="E31" s="6">
         <v>10</v>
       </c>
-      <c r="F31" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="10">
-        <f>IF(F31="NO","Oculto",IF(E31&lt;=0,"AGOTADO",IF(E31&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H31" s="11" t="s">
+      <c r="F31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Disponible</v>
+      </c>
+      <c r="H31" s="9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
+    <row r="32" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
         <v>78</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C32" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="7">
+      <c r="D32" s="5">
         <v>160000</v>
       </c>
-      <c r="E32" s="8">
+      <c r="E32" s="6">
         <v>2</v>
       </c>
-      <c r="F32" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="10">
-        <f>IF(F32="NO","Oculto",IF(E32&lt;=0,"AGOTADO",IF(E32&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H32" s="11" t="s">
+      <c r="F32" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>79</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G32"/>
+  <autoFilter ref="A4:G32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G32">
-    <cfRule type="containsText" dxfId="0" priority="1">
-      <formula>NOT(ISERROR(SEARCH("AGOTADO",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2">
-      <formula>NOT(ISERROR(SEARCH("Últimas",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3">
-      <formula>NOT(ISERROR(SEARCH("Oculto",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4">
-      <formula>NOT(ISERROR(SEARCH("Disponible",G5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E32">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E32" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F32">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F32" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{00000000-000E-0000-0000-000001000000}">
+            <xm:f>NOT(ISERROR(SEARCH("AGOTADO",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{00000000-000E-0000-0000-000002000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Últimas",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C6500"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{00000000-000E-0000-0000-000003000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Oculto",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF6B7472"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFEDEDED"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{00000000-000E-0000-0000-000004000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Disponible",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>G5:G32</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="13"/>
+      <c r="B1" s="20"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="12">
         <f>COUNTA(Inventario!$A$5:$A$32)</f>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Disponible")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Últimas unidades")</f>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"AGOTADO")</f>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Oculto")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="12">
         <f>SUM(Inventario!$E$5:$E$32)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="13">
         <f>SUMPRODUCT(Inventario!$D$5:$D$32,Inventario!$E$5:$E$32)</f>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+        <v>1990000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="14" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1820,145 +1922,145 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="10" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="17" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="10" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="10" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="10" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="17" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="10" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="10" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="10" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="17" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="10" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="10" t="s">
         <v>111</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizar inventario (14 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F2375B8-EDF5-492D-AC6D-4C8D76945E02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{621353CC-B20D-4F5D-A753-8466C39ED020}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1007,14 +1007,14 @@
         <v>170000</v>
       </c>
       <c r="E5" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="8" t="str">
         <f t="shared" ref="G5:G32" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H5" s="9" t="s">
         <v>14</v>
@@ -1034,7 +1034,7 @@
         <v>130000</v>
       </c>
       <c r="E6" s="6">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F6" s="7" t="s">
         <v>13</v>
@@ -1061,14 +1061,14 @@
         <v>120000</v>
       </c>
       <c r="E7" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>20</v>
@@ -1088,14 +1088,14 @@
         <v>130000</v>
       </c>
       <c r="E8" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>23</v>
@@ -1142,14 +1142,14 @@
         <v>130000</v>
       </c>
       <c r="E10" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F10" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H10" s="9" t="s">
         <v>27</v>
@@ -1169,14 +1169,14 @@
         <v>120000</v>
       </c>
       <c r="E11" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H11" s="9" t="s">
         <v>29</v>
@@ -1223,14 +1223,14 @@
         <v>160000</v>
       </c>
       <c r="E13" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H13" s="9" t="s">
         <v>35</v>
@@ -1304,14 +1304,14 @@
         <v>130000</v>
       </c>
       <c r="E16" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H16" s="9" t="s">
         <v>41</v>
@@ -1331,14 +1331,14 @@
         <v>200000</v>
       </c>
       <c r="E17" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G17" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H17" s="9" t="s">
         <v>43</v>
@@ -1385,14 +1385,14 @@
         <v>120000</v>
       </c>
       <c r="E19" s="6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H19" s="9" t="s">
         <v>47</v>
@@ -1412,14 +1412,14 @@
         <v>110000</v>
       </c>
       <c r="E20" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F20" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G20" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H20" s="9" t="s">
         <v>49</v>
@@ -1493,14 +1493,14 @@
         <v>140000</v>
       </c>
       <c r="E23" s="6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G23" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H23" s="9" t="s">
         <v>57</v>
@@ -1520,14 +1520,14 @@
         <v>130000</v>
       </c>
       <c r="E24" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F24" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G24" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H24" s="9" t="s">
         <v>60</v>
@@ -1547,14 +1547,14 @@
         <v>130000</v>
       </c>
       <c r="E25" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>AGOTADO</v>
+        <v>Últimas unidades</v>
       </c>
       <c r="H25" s="9" t="s">
         <v>62</v>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="B5" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Últimas unidades")</f>
-        <v>6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="B6" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"AGOTADO")</f>
-        <v>21</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="B8" s="12">
         <f>SUM(Inventario!$E$5:$E$32)</f>
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B9" s="13">
         <f>SUMPRODUCT(Inventario!$D$5:$D$32,Inventario!$E$5:$E$32)</f>
-        <v>2190000</v>
+        <v>5400000</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizar inventario (3 cambios)
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -1,14 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26F1DF04-64D2-4F9C-BE26-8B8C4B1D96B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Inventario" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Resumen" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Instrucciones" state="visible" r:id="rId6"/>
+    <sheet name="Inventario" sheetId="1" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" r:id="rId2"/>
+    <sheet name="Instrucciones" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -354,34 +374,34 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="&quot;$&quot; #,##0"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;\ #,##0"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <b/>
+      <sz val="16"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="16"/>
       <name val="Arial"/>
     </font>
     <font>
       <i/>
-      <color rgb="FF6b7472"/>
       <sz val="9"/>
+      <color rgb="FF6B7472"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -394,14 +414,14 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="8"/>
       <color rgb="FF9A9A9A"/>
-      <sz val="8"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="14"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -414,20 +434,20 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="9"/>
       <color rgb="FF9A9A9A"/>
-      <sz val="9"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="15"/>
       <color rgb="FFFFFFFF"/>
-      <sz val="15"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color rgb="FF2E8B80"/>
-      <sz val="11"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -478,12 +498,6 @@
   </cellStyleXfs>
   <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -514,7 +528,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="1" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -530,6 +543,13 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -537,11 +557,21 @@
   <dxfs count="4">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF6B7472"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFEDEDED"/>
         </patternFill>
       </fill>
     </dxf>
@@ -557,21 +587,11 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF6b7472"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FFEDEDED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -909,12 +929,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="52" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -925,893 +945,975 @@
     <col min="7" max="8" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+    </row>
+    <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="4" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+    </row>
+    <row r="4" spans="1:8" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+    <row r="5" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="5">
         <v>170000</v>
       </c>
-      <c r="E5" s="8">
+      <c r="E5" s="6">
         <v>2</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="10">
-        <f>IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H5" s="11" t="s">
+      <c r="F5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="8" t="str">
+        <f t="shared" ref="G5:G32" si="0">IF(F5="NO","Oculto",IF(E5&lt;=0,"AGOTADO",IF(E5&lt;=5,"Últimas unidades","Disponible")))</f>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+    <row r="6" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="7">
+      <c r="D6" s="5">
         <v>130000</v>
       </c>
-      <c r="E6" s="8">
-        <v>5</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="10">
-        <f>IF(F6="NO","Oculto",IF(E6&lt;=0,"AGOTADO",IF(E6&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H6" s="11" t="s">
+      <c r="E6" s="6">
+        <v>3</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H6" s="9" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
+    <row r="7" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="5">
         <v>130000</v>
       </c>
-      <c r="E7" s="8">
+      <c r="E7" s="6">
         <v>1</v>
       </c>
-      <c r="F7" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="10">
-        <f>IF(F7="NO","Oculto",IF(E7&lt;=0,"AGOTADO",IF(E7&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H7" s="11" t="s">
+      <c r="F7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+    <row r="8" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="5">
         <v>130000</v>
       </c>
-      <c r="E8" s="8">
+      <c r="E8" s="6">
         <v>1</v>
       </c>
-      <c r="F8" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="10">
-        <f>IF(F8="NO","Oculto",IF(E8&lt;=0,"AGOTADO",IF(E8&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H8" s="11" t="s">
+      <c r="F8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H8" s="9" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
+    <row r="9" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="5">
         <v>160000</v>
       </c>
-      <c r="E9" s="8">
+      <c r="E9" s="6">
         <v>0</v>
       </c>
-      <c r="F9" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G9" s="10">
-        <f>IF(F9="NO","Oculto",IF(E9&lt;=0,"AGOTADO",IF(E9&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H9" s="11" t="s">
+      <c r="F9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+    <row r="10" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="5">
         <v>130000</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="6">
         <v>2</v>
       </c>
-      <c r="F10" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G10" s="10">
-        <f>IF(F10="NO","Oculto",IF(E10&lt;=0,"AGOTADO",IF(E10&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H10" s="11" t="s">
+      <c r="F10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H10" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+    <row r="11" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="5">
         <v>120000</v>
       </c>
-      <c r="E11" s="8">
+      <c r="E11" s="6">
+        <v>1</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="5">
+        <v>160000</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="5">
+        <v>160000</v>
+      </c>
+      <c r="E13" s="6">
+        <v>1</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="5">
+        <v>160000</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="5">
+        <v>200000</v>
+      </c>
+      <c r="E15" s="6">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="5">
+        <v>130000</v>
+      </c>
+      <c r="E16" s="6">
+        <v>1</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G16" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="5">
+        <v>200000</v>
+      </c>
+      <c r="E17" s="6">
+        <v>1</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G17" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="5">
+        <v>130000</v>
+      </c>
+      <c r="E18" s="6">
+        <v>0</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="5">
+        <v>120000</v>
+      </c>
+      <c r="E19" s="6">
+        <v>4</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="5">
+        <v>110000</v>
+      </c>
+      <c r="E20" s="6">
         <v>2</v>
       </c>
-      <c r="F11" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="10">
-        <f>IF(F11="NO","Oculto",IF(E11&lt;=0,"AGOTADO",IF(E11&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="4" t="s">
+      <c r="F20" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C21" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="7">
+      <c r="D21" s="5">
+        <v>120000</v>
+      </c>
+      <c r="E21" s="6">
+        <v>0</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="5">
+        <v>120000</v>
+      </c>
+      <c r="E22" s="6">
+        <v>0</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="5">
+        <v>140000</v>
+      </c>
+      <c r="E23" s="6">
+        <v>2</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D24" s="5">
+        <v>130000</v>
+      </c>
+      <c r="E24" s="6">
+        <v>1</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G24" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="5">
+        <v>130000</v>
+      </c>
+      <c r="E25" s="6">
+        <v>1</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D26" s="5">
+        <v>140000</v>
+      </c>
+      <c r="E26" s="6">
+        <v>3</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D27" s="5">
+        <v>130000</v>
+      </c>
+      <c r="E27" s="6">
+        <v>1</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H27" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" s="2" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" s="5">
+        <v>120000</v>
+      </c>
+      <c r="E28" s="6">
+        <v>0</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G28" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>AGOTADO</v>
+      </c>
+      <c r="H28" s="9" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D29" s="5">
+        <v>140000</v>
+      </c>
+      <c r="E29" s="6">
+        <v>1</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G29" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H29" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="5">
         <v>160000</v>
       </c>
-      <c r="E12" s="8">
-        <v>0</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G12" s="10">
-        <f>IF(F12="NO","Oculto",IF(E12&lt;=0,"AGOTADO",IF(E12&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C13" s="6" t="s">
+      <c r="E30" s="6">
+        <v>2</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G30" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H30" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="5">
+        <v>60000</v>
+      </c>
+      <c r="E31" s="6">
+        <v>10</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G31" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Disponible</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" s="2" customFormat="1" ht="12.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="7">
+      <c r="D32" s="5">
         <v>160000</v>
       </c>
-      <c r="E13" s="8">
+      <c r="E32" s="6">
         <v>1</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G13" s="10">
-        <f>IF(F13="NO","Oculto",IF(E13&lt;=0,"AGOTADO",IF(E13&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="7">
-        <v>160000</v>
-      </c>
-      <c r="E14" s="8">
-        <v>0</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G14" s="10">
-        <f>IF(F14="NO","Oculto",IF(E14&lt;=0,"AGOTADO",IF(E14&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D15" s="7">
-        <v>200000</v>
-      </c>
-      <c r="E15" s="8">
-        <v>0</v>
-      </c>
-      <c r="F15" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="10">
-        <f>IF(F15="NO","Oculto",IF(E15&lt;=0,"AGOTADO",IF(E15&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H15" s="11" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="7">
-        <v>130000</v>
-      </c>
-      <c r="E16" s="8">
-        <v>1</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G16" s="10">
-        <f>IF(F16="NO","Oculto",IF(E16&lt;=0,"AGOTADO",IF(E16&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="7">
-        <v>200000</v>
-      </c>
-      <c r="E17" s="8">
-        <v>1</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G17" s="10">
-        <f>IF(F17="NO","Oculto",IF(E17&lt;=0,"AGOTADO",IF(E17&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D18" s="7">
-        <v>130000</v>
-      </c>
-      <c r="E18" s="8">
-        <v>0</v>
-      </c>
-      <c r="F18" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G18" s="10">
-        <f>IF(F18="NO","Oculto",IF(E18&lt;=0,"AGOTADO",IF(E18&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="7">
-        <v>120000</v>
-      </c>
-      <c r="E19" s="8">
-        <v>4</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="10">
-        <f>IF(F19="NO","Oculto",IF(E19&lt;=0,"AGOTADO",IF(E19&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="7">
-        <v>110000</v>
-      </c>
-      <c r="E20" s="8">
-        <v>2</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="10">
-        <f>IF(F20="NO","Oculto",IF(E20&lt;=0,"AGOTADO",IF(E20&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H20" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="7">
-        <v>120000</v>
-      </c>
-      <c r="E21" s="8">
-        <v>0</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="10">
-        <f>IF(F21="NO","Oculto",IF(E21&lt;=0,"AGOTADO",IF(E21&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="7">
-        <v>120000</v>
-      </c>
-      <c r="E22" s="8">
-        <v>0</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="10">
-        <f>IF(F22="NO","Oculto",IF(E22&lt;=0,"AGOTADO",IF(E22&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H22" s="11" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D23" s="7">
-        <v>140000</v>
-      </c>
-      <c r="E23" s="8">
-        <v>2</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="10">
-        <f>IF(F23="NO","Oculto",IF(E23&lt;=0,"AGOTADO",IF(E23&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H23" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" s="7">
-        <v>130000</v>
-      </c>
-      <c r="E24" s="8">
-        <v>1</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G24" s="10">
-        <f>IF(F24="NO","Oculto",IF(E24&lt;=0,"AGOTADO",IF(E24&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H24" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="7">
-        <v>130000</v>
-      </c>
-      <c r="E25" s="8">
-        <v>1</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="10">
-        <f>IF(F25="NO","Oculto",IF(E25&lt;=0,"AGOTADO",IF(E25&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H25" s="11" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D26" s="7">
-        <v>140000</v>
-      </c>
-      <c r="E26" s="8">
-        <v>3</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="10">
-        <f>IF(F26="NO","Oculto",IF(E26&lt;=0,"AGOTADO",IF(E26&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H26" s="11" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D27" s="7">
-        <v>130000</v>
-      </c>
-      <c r="E27" s="8">
-        <v>1</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="10">
-        <f>IF(F27="NO","Oculto",IF(E27&lt;=0,"AGOTADO",IF(E27&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H27" s="11" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D28" s="7">
-        <v>120000</v>
-      </c>
-      <c r="E28" s="8">
-        <v>0</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="10">
-        <f>IF(F28="NO","Oculto",IF(E28&lt;=0,"AGOTADO",IF(E28&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H28" s="11" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="7">
-        <v>140000</v>
-      </c>
-      <c r="E29" s="8">
-        <v>1</v>
-      </c>
-      <c r="F29" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G29" s="10">
-        <f>IF(F29="NO","Oculto",IF(E29&lt;=0,"AGOTADO",IF(E29&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H29" s="11" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="7">
-        <v>160000</v>
-      </c>
-      <c r="E30" s="8">
-        <v>2</v>
-      </c>
-      <c r="F30" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G30" s="10">
-        <f>IF(F30="NO","Oculto",IF(E30&lt;=0,"AGOTADO",IF(E30&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H30" s="11" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D31" s="7">
-        <v>60000</v>
-      </c>
-      <c r="E31" s="8">
-        <v>10</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G31" s="10">
-        <f>IF(F31="NO","Oculto",IF(E31&lt;=0,"AGOTADO",IF(E31&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H31" s="11" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="D32" s="7">
-        <v>160000</v>
-      </c>
-      <c r="E32" s="8">
-        <v>2</v>
-      </c>
-      <c r="F32" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G32" s="10">
-        <f>IF(F32="NO","Oculto",IF(E32&lt;=0,"AGOTADO",IF(E32&lt;=5,"Últimas unidades","Disponible")))</f>
-      </c>
-      <c r="H32" s="11" t="s">
+      <c r="F32" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G32" s="8" t="str">
+        <f t="shared" si="0"/>
+        <v>Últimas unidades</v>
+      </c>
+      <c r="H32" s="9" t="s">
         <v>79</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G32"/>
+  <autoFilter ref="A4:G32" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="G5:G32">
-    <cfRule type="containsText" dxfId="0" priority="1">
-      <formula>NOT(ISERROR(SEARCH("AGOTADO",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="2">
-      <formula>NOT(ISERROR(SEARCH("Últimas",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3">
-      <formula>NOT(ISERROR(SEARCH("Oculto",G5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4">
-      <formula>NOT(ISERROR(SEARCH("Disponible",G5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E32">
+    <dataValidation type="whole" operator="greaterThanOrEqual" showErrorMessage="1" errorTitle="Cantidad inválida" error="Escribe un número entero de 0 en adelante." sqref="E5:E32" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F32">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="Valor inválido" error="Escribe SI o NO." sqref="F5:F32" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="1" operator="containsText" id="{00000000-000E-0000-0000-000001000000}">
+            <xm:f>NOT(ISERROR(SEARCH("AGOTADO",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="2" operator="containsText" id="{00000000-000E-0000-0000-000002000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Últimas",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C6500"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="3" operator="containsText" id="{00000000-000E-0000-0000-000003000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Oculto",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF6B7472"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFEDEDED"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <x14:cfRule type="containsText" priority="4" operator="containsText" id="{00000000-000E-0000-0000-000004000000}">
+            <xm:f>NOT(ISERROR(SEARCH("Disponible",G5)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>G5:G32</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B13"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+    <row r="1" spans="1:2" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="13"/>
+      <c r="B1" s="20"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="15">
+      <c r="B3" s="12">
         <f>COUNTA(Inventario!$A$5:$A$32)</f>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="B4" s="15">
+      <c r="B4" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Disponible")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="B5" s="15">
+      <c r="B5" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Últimas unidades")</f>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="B6" s="15">
+      <c r="B6" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"AGOTADO")</f>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B7" s="15">
+      <c r="B7" s="12">
         <f>COUNTIF(Inventario!$G$5:$G$32,"Oculto")</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="A8" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="15">
+      <c r="B8" s="12">
         <f>SUM(Inventario!$E$5:$E$32)</f>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="B9" s="16">
+      <c r="B9" s="13">
         <f>SUMPRODUCT(Inventario!$D$5:$D$32,Inventario!$E$5:$E$32)</f>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="17" t="s">
+        <v>4870000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="14" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="18" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="15" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1820,145 +1922,145 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A25"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="16" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="10" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="10" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
+      <c r="A9" s="17" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="10" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="10" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="10" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="10" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="10" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="A16" s="17" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="10" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="10" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="10" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="10" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="10" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="20" t="s">
+      <c r="A22" s="17" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="10" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="10" t="s">
         <v>111</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>